<commit_message>
Poprawki matura maj 2026
</commit_message>
<xml_diff>
--- a/Matura maj 2026/zad7.xlsx
+++ b/Matura maj 2026/zad7.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gosia\Desktop\Matura 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{697E6447-A196-4F72-A046-1A3643ED2443}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C5AE2A1-DF5A-4044-8AE0-D51DFE1AD098}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="14400" activeTab="4" xr2:uid="{AFE5701C-A157-4FAC-90E0-63C110A2425A}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="14400" activeTab="1" xr2:uid="{AFE5701C-A157-4FAC-90E0-63C110A2425A}"/>
   </bookViews>
   <sheets>
     <sheet name="Wykres 71" sheetId="4" r:id="rId1"/>
@@ -105,9 +105,6 @@
     <t>gru</t>
   </si>
   <si>
-    <t>Suma z Temp</t>
-  </si>
-  <si>
     <t>osobno dla miesiąca</t>
   </si>
   <si>
@@ -142,6 +139,9 @@
   </si>
   <si>
     <t>lp</t>
+  </si>
+  <si>
+    <t>Średnia z Temp</t>
   </si>
 </sst>
 </file>
@@ -490,40 +490,40 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>33.600000000000009</c:v>
+                  <c:v>1.0838709677419358</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>115.9</c:v>
+                  <c:v>4.1392857142857142</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>125.70000000000002</c:v>
+                  <c:v>4.0548387096774201</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>221.1</c:v>
+                  <c:v>7.37</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>491.80000000000007</c:v>
+                  <c:v>15.86451612903226</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>614.59999999999991</c:v>
+                  <c:v>20.486666666666665</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>632.20000000000016</c:v>
+                  <c:v>20.393548387096779</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>655.1</c:v>
+                  <c:v>21.13225806451613</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>410.10000000000008</c:v>
+                  <c:v>13.670000000000003</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>386.8</c:v>
+                  <c:v>12.477419354838711</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>156</c:v>
+                  <c:v>5.2</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>49.3</c:v>
+                  <c:v>1.5903225806451613</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -662,37 +662,6 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
-    <c:legend>
-      <c:legendPos val="r"/>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="pl-PL"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
@@ -735,7 +704,6 @@
         <c14:dropZoneFilter val="1"/>
         <c14:dropZoneCategories val="1"/>
         <c14:dropZoneData val="1"/>
-        <c14:dropZoneSeries val="1"/>
         <c14:dropZonesVisible val="1"/>
       </c14:pivotOptions>
     </c:ext>
@@ -6621,7 +6589,7 @@
     <i/>
   </colItems>
   <dataFields count="1">
-    <dataField name="Suma z Temp" fld="1" baseField="3" baseItem="1" numFmtId="164"/>
+    <dataField name="Średnia z Temp" fld="1" subtotal="average" baseField="3" baseItem="1" numFmtId="164"/>
   </dataFields>
   <chartFormats count="1">
     <chartFormat chart="2" format="1" series="1">
@@ -7056,7 +7024,7 @@
   <cols>
     <col min="1" max="1" width="10.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="16.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -7095,7 +7063,7 @@
         <v>3</v>
       </c>
       <c r="H3" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
@@ -7112,7 +7080,7 @@
         <v>5</v>
       </c>
       <c r="H4" s="4">
-        <v>33.600000000000009</v>
+        <v>1.0838709677419358</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
@@ -7129,7 +7097,7 @@
         <v>6</v>
       </c>
       <c r="H5" s="4">
-        <v>115.9</v>
+        <v>4.1392857142857142</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
@@ -7146,7 +7114,7 @@
         <v>7</v>
       </c>
       <c r="H6" s="4">
-        <v>125.70000000000002</v>
+        <v>4.0548387096774201</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
@@ -7163,7 +7131,7 @@
         <v>8</v>
       </c>
       <c r="H7" s="4">
-        <v>221.1</v>
+        <v>7.37</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
@@ -7180,7 +7148,7 @@
         <v>9</v>
       </c>
       <c r="H8" s="4">
-        <v>491.80000000000007</v>
+        <v>15.86451612903226</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
@@ -7197,7 +7165,7 @@
         <v>10</v>
       </c>
       <c r="H9" s="4">
-        <v>614.59999999999991</v>
+        <v>20.486666666666665</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
@@ -7214,7 +7182,7 @@
         <v>11</v>
       </c>
       <c r="H10" s="4">
-        <v>632.20000000000016</v>
+        <v>20.393548387096779</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
@@ -7231,7 +7199,7 @@
         <v>12</v>
       </c>
       <c r="H11" s="4">
-        <v>655.1</v>
+        <v>21.13225806451613</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
@@ -7248,7 +7216,7 @@
         <v>13</v>
       </c>
       <c r="H12" s="4">
-        <v>410.10000000000008</v>
+        <v>13.670000000000003</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
@@ -7265,7 +7233,7 @@
         <v>14</v>
       </c>
       <c r="H13" s="4">
-        <v>386.8</v>
+        <v>12.477419354838711</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
@@ -7282,7 +7250,7 @@
         <v>15</v>
       </c>
       <c r="H14" s="4">
-        <v>156</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
@@ -7299,7 +7267,7 @@
         <v>16</v>
       </c>
       <c r="H15" s="4">
-        <v>49.3</v>
+        <v>1.5903225806451613</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
@@ -7316,7 +7284,7 @@
         <v>4</v>
       </c>
       <c r="H16" s="4">
-        <v>3892.2000000000003</v>
+        <v>10.663561643835619</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -11194,7 +11162,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -11203,7 +11171,7 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
@@ -11246,7 +11214,7 @@
         <v>3</v>
       </c>
       <c r="L3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
@@ -17403,7 +17371,7 @@
         <v>0</v>
       </c>
       <c r="E323">
-        <f t="shared" ref="E323:E386" si="11">IF(B322&lt;&gt;B323,IF(D323=0,1,0),IF(D323=0,E322+1,0))</f>
+        <f t="shared" ref="E323:E366" si="11">IF(B322&lt;&gt;B323,IF(D323=0,1,0),IF(D323=0,E322+1,0))</f>
         <v>1</v>
       </c>
     </row>
@@ -18242,35 +18210,35 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" t="s">
         <v>23</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>24</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>25</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>26</v>
-      </c>
-      <c r="H1" t="s">
-        <v>27</v>
       </c>
       <c r="I1">
         <f>75%*10000</f>
         <v>7500</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="M1" s="5">
         <v>80</v>
@@ -18379,7 +18347,7 @@
         <v>1949.5563750000001</v>
       </c>
       <c r="H4">
-        <f t="shared" ref="H3:H66" si="8">G4*1.75%</f>
+        <f t="shared" ref="H4:H66" si="8">G4*1.75%</f>
         <v>34.117236562500004</v>
       </c>
       <c r="I4" t="str">
@@ -25285,28 +25253,28 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" t="s">
         <v>23</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>24</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>25</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>26</v>
-      </c>
-      <c r="H1" t="s">
-        <v>27</v>
       </c>
       <c r="I1">
         <v>5000</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="M1" s="5">
         <v>94</v>
@@ -25347,7 +25315,7 @@
         <v>0</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="M2">
         <f>SUM(I2:I185)</f>

</xml_diff>